<commit_message>
refactor: restructure PI configuration files
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/ProjectConfiguration.xlsx
+++ b/inst/extdata/examples/TestProject/ProjectConfiguration.xlsx
@@ -1,41 +1,167 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR\inst\extdata\examples\TestProject\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39E34A44-10F5-4695-AB23-231277161660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="2500" yWindow="1580" windowWidth="34360" windowHeight="19040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+  <si>
+    <t>Property</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>modelFolder</t>
+  </si>
+  <si>
+    <t>Models/Simulations/</t>
+  </si>
+  <si>
+    <t>Path to the folder with pkml simulation files; relative to the location of this file</t>
+  </si>
+  <si>
+    <t>configurationsFolder</t>
+  </si>
+  <si>
+    <t>Configurations/</t>
+  </si>
+  <si>
+    <t>Path to the folder with excel files with parametrization; relative to the location of this file</t>
+  </si>
+  <si>
+    <t>modelParamsFile</t>
+  </si>
+  <si>
+    <t>ModelParameters.xlsx</t>
+  </si>
+  <si>
+    <t>Name of the excel file with global model parametrization. Must be located in the "paramsFolder"</t>
+  </si>
+  <si>
+    <t>individualsFile</t>
+  </si>
+  <si>
+    <t>Individuals.xlsx</t>
+  </si>
+  <si>
+    <t>Name of the excel file with individual-specific model parametrization. Must be located in the "paramsFolder"</t>
+  </si>
+  <si>
+    <t>populationsFile</t>
+  </si>
+  <si>
+    <t>Populations.xlsx</t>
+  </si>
+  <si>
+    <t>Name of the excel file with population information. Must be located in the "paramsFolder"</t>
+  </si>
+  <si>
+    <t>populationsFolder</t>
+  </si>
+  <si>
+    <t>PopulationsCSV</t>
+  </si>
+  <si>
+    <t>Name of the folder containing population defined in files</t>
+  </si>
+  <si>
+    <t>scenariosFile</t>
+  </si>
+  <si>
+    <t>Scenarios.xlsx</t>
+  </si>
+  <si>
+    <t>Name of the excel file with scenario definitions. Must be located in the "paramsFolder"</t>
+  </si>
+  <si>
+    <t>applicationsFile</t>
+  </si>
+  <si>
+    <t>Applications.xlsx</t>
+  </si>
+  <si>
+    <t>Name of the excel file scenario-specific parameters such as application protocol parameters. Must be located in the "paramsFolder"</t>
+  </si>
+  <si>
+    <t>plotsFile</t>
+  </si>
+  <si>
+    <t>Plots.xlsx</t>
+  </si>
+  <si>
+    <t>Name of the excel file with plot definitions. Must be located in the "paramsFolder"</t>
+  </si>
+  <si>
+    <t>parameterIdentificationFile</t>
+  </si>
+  <si>
+    <t>ParameterIdentification.xlsx</t>
+  </si>
+  <si>
+    <t>dataFolder</t>
+  </si>
+  <si>
+    <t>Data/</t>
+  </si>
+  <si>
+    <t>Path to the folder where experimental data files are located; relative to the location of this file</t>
+  </si>
+  <si>
+    <t>dataFile</t>
+  </si>
+  <si>
+    <t>TestProject_TimeValuesData.xlsx</t>
+  </si>
+  <si>
+    <t>Name of the excel file with experimental data. Must be located in the "dataFolder"</t>
+  </si>
+  <si>
+    <t>dataImporterConfigurationFile</t>
+  </si>
+  <si>
+    <t>esqlabs_dataImporter_configuration.xml</t>
+  </si>
+  <si>
+    <t>Name of data importer configuration file in xml format used to load the data. Must be located in the "dataFolder"</t>
+  </si>
+  <si>
+    <t>outputFolder</t>
+  </si>
+  <si>
+    <t>Results/</t>
+  </si>
+  <si>
+    <t>Path to the folder where the results should be saved to; relative to the location of this file</t>
+  </si>
+  <si>
+    <t>Name of the excel file with parameter identification task definitions. Must be located in the "configurationsFolder"</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +191,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,188 +530,183 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.9140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Property</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Description</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>modelFolder</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Models/Simulations/</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Path to the folder with pkml simulation files; relative to the location of this file</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>configurationsFolder</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Configurations/</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Path to the folder with excel files with parametrization; relative to the location of this file</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>modelParamsFile</v>
-      </c>
-      <c r="B4" t="str">
-        <v>ModelParameters.xlsx</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Name of the excel file with global model parametrization. Must be located in the "paramsFolder"</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>individualsFile</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Individuals.xlsx</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Name of the excel file with individual-specific model parametrization. Must be located in the "paramsFolder"</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>populationsFile</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Populations.xlsx</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Name of the excel file with population information. Must be located in the "paramsFolder"</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>populationsFolder</v>
-      </c>
-      <c r="B7" t="str">
-        <v>PopulationsCSV</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Name of the folder containing population defined in files</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>scenariosFile</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Scenarios.xlsx</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Name of the excel file with scenario definitions. Must be located in the "paramsFolder"</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>applicationsFile</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Applications.xlsx</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Name of the excel file scenario-specific parameters such as application protocol parameters. Must be located in the "paramsFolder"</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>plotsFile</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Plots.xlsx</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Name of the excel file with plot definitions. Must be located in the "paramsFolder"</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>analysisFolder</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Analysis/</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Path to the folder containing excel files with analysis task definitions; relative to the location of this file</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>parameterIdentificationFile</v>
-      </c>
-      <c r="B12" t="str">
-        <v>ParameterIdentification.xlsx</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Name of the excel file with parameter identification task definitions. Must be located in the "analysesFolder"</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>dataFolder</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Data/</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Path to the folder where experimental data files are located; relative to the location of this file</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>dataFile</v>
-      </c>
-      <c r="B14" t="str">
-        <v>TestProject_TimeValuesData.xlsx</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Name of the excel file with experimental data. Must be located in the "dataFolder"</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>dataImporterConfigurationFile</v>
-      </c>
-      <c r="B15" t="str">
-        <v>esqlabs_dataImporter_configuration.xml</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Name of data importer configuration file in xml format used to load the data. Must be located in the "dataFolder"</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>outputFolder</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Results/</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Path to the folder where the results should be saved to; relative to the location of this file</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
+    <ignoredError sqref="A1:C10 A12:C15 A11:B11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: fix incorrect path in configuration description
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/ProjectConfiguration.xlsx
+++ b/inst/extdata/examples/TestProject/ProjectConfiguration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR\inst\extdata\examples\TestProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39E34A44-10F5-4695-AB23-231277161660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7AE1E29-BC24-4D57-A06B-E3435808FAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2500" yWindow="1580" windowWidth="34360" windowHeight="19040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2830" yWindow="1200" windowWidth="34360" windowHeight="19040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -55,27 +55,18 @@
     <t>ModelParameters.xlsx</t>
   </si>
   <si>
-    <t>Name of the excel file with global model parametrization. Must be located in the "paramsFolder"</t>
-  </si>
-  <si>
     <t>individualsFile</t>
   </si>
   <si>
     <t>Individuals.xlsx</t>
   </si>
   <si>
-    <t>Name of the excel file with individual-specific model parametrization. Must be located in the "paramsFolder"</t>
-  </si>
-  <si>
     <t>populationsFile</t>
   </si>
   <si>
     <t>Populations.xlsx</t>
   </si>
   <si>
-    <t>Name of the excel file with population information. Must be located in the "paramsFolder"</t>
-  </si>
-  <si>
     <t>populationsFolder</t>
   </si>
   <si>
@@ -91,27 +82,18 @@
     <t>Scenarios.xlsx</t>
   </si>
   <si>
-    <t>Name of the excel file with scenario definitions. Must be located in the "paramsFolder"</t>
-  </si>
-  <si>
     <t>applicationsFile</t>
   </si>
   <si>
     <t>Applications.xlsx</t>
   </si>
   <si>
-    <t>Name of the excel file scenario-specific parameters such as application protocol parameters. Must be located in the "paramsFolder"</t>
-  </si>
-  <si>
     <t>plotsFile</t>
   </si>
   <si>
     <t>Plots.xlsx</t>
   </si>
   <si>
-    <t>Name of the excel file with plot definitions. Must be located in the "paramsFolder"</t>
-  </si>
-  <si>
     <t>parameterIdentificationFile</t>
   </si>
   <si>
@@ -155,6 +137,24 @@
   </si>
   <si>
     <t>Name of the excel file with parameter identification task definitions. Must be located in the "configurationsFolder"</t>
+  </si>
+  <si>
+    <t>Name of the excel file with global model parametrization. Must be located in the "configurationsFolder"</t>
+  </si>
+  <si>
+    <t>Name of the excel file with individual-specific model parametrization. Must be located in the "configurationsFolder"</t>
+  </si>
+  <si>
+    <t>Name of the excel file with population information. Must be located in the "configurationsFolder"</t>
+  </si>
+  <si>
+    <t>Name of the excel file with scenario definitions. Must be located in the "configurationsFolder"</t>
+  </si>
+  <si>
+    <t>Name of the excel file scenario-specific parameters such as application protocol parameters. Must be located in the "configurationsFolder"</t>
+  </si>
+  <si>
+    <t>Name of the excel file with plot definitions. Must be located in the "configurationsFolder"</t>
   </si>
 </sst>
 </file>
@@ -579,134 +579,134 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C10 A12:C15 A11:B11" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C3 A12:C15 A11:B11 A7:C7 A4:B4 A5:B5 A6:B6 A10:B10 A8:B8 A9:B9" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>